<commit_message>
Successfully merged all Datasets and removed any found contamination
</commit_message>
<xml_diff>
--- a/CDC Annotatie.xlsx
+++ b/CDC Annotatie.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20409"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Desktop\Stage VIB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\irc\Desktop\Interschip Bioinformatis 2025-2026\DC-Atlas-VIB-Scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54AEA024-2CFF-4ECD-9CC7-3487B5FBD06F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B590E6AA-8982-4433-92F5-0357F4D8E676}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -114,9 +114,6 @@
     <t>Cd3d,Cd4,S100a4,Ccr10,Il7r</t>
   </si>
   <si>
-    <t>Cd3d,Cd4, Il2ra,Foxp3</t>
-  </si>
-  <si>
     <t>T reg</t>
   </si>
   <si>
@@ -166,6 +163,9 @@
   </si>
   <si>
     <t>Mcpt8,Mcemp1</t>
+  </si>
+  <si>
+    <t>Cd3d,Cd4,Il2ra,Foxp3</t>
   </si>
 </sst>
 </file>
@@ -248,7 +248,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -561,16 +561,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" customWidth="1"/>
-    <col min="2" max="2" width="35.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="214.6640625" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" customWidth="1"/>
+    <col min="1" max="1" width="13.5234375" customWidth="1"/>
+    <col min="2" max="2" width="35.89453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="214.68359375" customWidth="1"/>
+    <col min="4" max="4" width="27.1015625" customWidth="1"/>
     <col min="5" max="5" width="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -587,7 +587,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -598,7 +598,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -609,7 +609,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -620,7 +620,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -631,7 +631,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -642,7 +642,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -653,7 +653,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -664,7 +664,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -675,7 +675,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
@@ -686,7 +686,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
@@ -697,7 +697,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="2" t="s">
         <v>3</v>
       </c>
@@ -708,115 +708,115 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C13" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" t="s">
         <v>32</v>
       </c>
-      <c r="C15" t="s">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" t="s">
         <v>34</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" t="s">
         <v>36</v>
       </c>
-      <c r="C17" t="s">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" t="s">
         <v>38</v>
       </c>
-      <c r="C18" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" t="s">
         <v>40</v>
       </c>
-      <c r="C19" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" t="s">
         <v>42</v>
       </c>
-      <c r="C20" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" t="s">
         <v>44</v>
       </c>
-      <c r="C21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B22" s="5"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B23" s="5"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B24" s="5"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B25" s="5"/>
     </row>
   </sheetData>

</xml_diff>